<commit_message>
Fix Excel charts and add the data model to the README
- Bar charts start at zero (a truncated axis exaggerated a few dollars of difference)
- Line chart is unsmoothed and shows a legend
- Axes are explicitly enabled so Excel displays them
- Sheets print on one page width
- README: data model section
</commit_message>
<xml_diff>
--- a/reports/sales_analysis.xlsx
+++ b/reports/sales_analysis.xlsx
@@ -210,6 +210,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -220,7 +221,9 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -301,6 +304,7 @@
               <f>'monthly_revenue'!$C$2:$C$61</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="1"/>
@@ -333,6 +337,7 @@
               <f>'monthly_revenue'!$D$2:$D$61</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -342,6 +347,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -352,7 +358,9 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -439,6 +447,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -449,7 +458,9 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -533,6 +544,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -543,7 +555,9 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -967,7 +981,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1124,6 +1138,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1131,7 +1146,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1566,6 +1581,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1573,7 +1589,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1656,6 +1672,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1663,7 +1680,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1817,6 +1834,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -1825,7 +1843,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2820,6 +2838,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -2828,7 +2847,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4291,6 +4310,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -4298,7 +4318,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4873,6 +4893,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -4881,7 +4902,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -5378,6 +5399,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -5386,7 +5408,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -7280,6 +7302,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -7287,7 +7310,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -7517,6 +7540,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -7524,7 +7548,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -7799,5 +7823,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(sql): score RFM with PERCENT_RANK so ties share a score; vendor and pin the Chinook database
NTILE split customers with identical behaviour into different bands by CustomerId. PERCENT_RANK gives
equal values equal scores, so Frequency (58 of 59 customers have the same invoice count) is now constant
instead of an arbitrary spread, and the segments are 4 high, 29 middle, 26 low. Tests check that equal
values get equal scores. The 1 MB MIT-licensed database is included with its licence and pinned by SHA-256,
so tests and CI need no network; a weekly workflow checks that upstream is unchanged.
</commit_message>
<xml_diff>
--- a/reports/sales_analysis.xlsx
+++ b/reports/sales_analysis.xlsx
@@ -5473,28 +5473,28 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C2" t="n">
         <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>45.62</v>
+        <v>49.62</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -5504,28 +5504,28 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="C3" t="n">
         <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>41.62</v>
+        <v>45.62</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -5535,28 +5535,28 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B4" t="n">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C4" t="n">
         <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>39.62</v>
+        <v>42.62</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -5566,28 +5566,28 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" t="n">
-        <v>155</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
         <v>7</v>
       </c>
       <c r="D5" t="n">
-        <v>45.62</v>
+        <v>41.62</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
         <v>3</v>
       </c>
       <c r="H5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -5597,264 +5597,264 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
+        <v>155</v>
       </c>
       <c r="C6" t="n">
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>42.62</v>
+        <v>45.62</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
         <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="B7" t="n">
-        <v>199</v>
+        <v>124</v>
       </c>
       <c r="C7" t="n">
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>40.62</v>
+        <v>43.62</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="B8" t="n">
-        <v>101</v>
+        <v>217</v>
       </c>
       <c r="C8" t="n">
         <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>40.62</v>
+        <v>43.62</v>
       </c>
       <c r="E8" t="n">
         <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="B9" t="n">
-        <v>31</v>
+        <v>202</v>
       </c>
       <c r="C9" t="n">
         <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>39.62</v>
+        <v>43.62</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
         <v>3</v>
       </c>
       <c r="H9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="C10" t="n">
         <v>7</v>
       </c>
       <c r="D10" t="n">
-        <v>38.62</v>
+        <v>42.62</v>
       </c>
       <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
         <v>3</v>
       </c>
-      <c r="F10" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" t="n">
-        <v>2</v>
-      </c>
       <c r="H10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="B11" t="n">
-        <v>62</v>
+        <v>230</v>
       </c>
       <c r="C11" t="n">
         <v>7</v>
       </c>
       <c r="D11" t="n">
-        <v>37.62</v>
+        <v>40.62</v>
       </c>
       <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
         <v>3</v>
       </c>
-      <c r="F11" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2</v>
-      </c>
       <c r="H11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B12" t="n">
-        <v>47</v>
+        <v>199</v>
       </c>
       <c r="C12" t="n">
         <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>37.62</v>
+        <v>40.62</v>
       </c>
       <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
         <v>3</v>
       </c>
-      <c r="F12" t="n">
-        <v>3</v>
-      </c>
-      <c r="G12" t="n">
-        <v>2</v>
-      </c>
       <c r="H12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B13" t="n">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="C13" t="n">
         <v>7</v>
       </c>
       <c r="D13" t="n">
-        <v>37.62</v>
+        <v>40.62</v>
       </c>
       <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="n">
         <v>3</v>
       </c>
-      <c r="F13" t="n">
-        <v>3</v>
-      </c>
-      <c r="G13" t="n">
-        <v>2</v>
-      </c>
       <c r="H13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B14" t="n">
-        <v>39</v>
+        <v>93</v>
       </c>
       <c r="C14" t="n">
         <v>7</v>
       </c>
       <c r="D14" t="n">
-        <v>49.62</v>
+        <v>39.62</v>
       </c>
       <c r="E14" t="n">
         <v>3</v>
@@ -5863,289 +5863,289 @@
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B15" t="n">
-        <v>434</v>
+        <v>80</v>
       </c>
       <c r="C15" t="n">
         <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>46.62</v>
+        <v>39.62</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B16" t="n">
-        <v>124</v>
+        <v>31</v>
       </c>
       <c r="C16" t="n">
         <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>43.62</v>
+        <v>39.62</v>
       </c>
       <c r="E16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
         <v>2</v>
       </c>
-      <c r="F16" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" t="n">
-        <v>3</v>
-      </c>
       <c r="H16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="B17" t="n">
-        <v>217</v>
+        <v>49</v>
       </c>
       <c r="C17" t="n">
         <v>7</v>
       </c>
       <c r="D17" t="n">
-        <v>43.62</v>
+        <v>39.62</v>
       </c>
       <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
         <v>2</v>
       </c>
-      <c r="F17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" t="n">
-        <v>3</v>
-      </c>
       <c r="H17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>37</v>
+        <v>58</v>
       </c>
       <c r="B18" t="n">
-        <v>202</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
         <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>43.62</v>
+        <v>38.62</v>
       </c>
       <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="n">
         <v>2</v>
       </c>
-      <c r="F18" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" t="n">
-        <v>3</v>
-      </c>
       <c r="H18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B19" t="n">
-        <v>168</v>
+        <v>261</v>
       </c>
       <c r="C19" t="n">
         <v>7</v>
       </c>
       <c r="D19" t="n">
-        <v>39.62</v>
+        <v>47.62</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
         <v>3</v>
       </c>
       <c r="H19" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B20" t="n">
-        <v>248</v>
+        <v>434</v>
       </c>
       <c r="C20" t="n">
         <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>37.62</v>
+        <v>46.62</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
         <v>3</v>
       </c>
-      <c r="G20" t="n">
-        <v>2</v>
-      </c>
       <c r="H20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="B21" t="n">
-        <v>194</v>
+        <v>137</v>
       </c>
       <c r="C21" t="n">
         <v>7</v>
       </c>
       <c r="D21" t="n">
-        <v>37.62</v>
+        <v>39.62</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
       </c>
       <c r="H21" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="B22" t="n">
-        <v>140</v>
+        <v>168</v>
       </c>
       <c r="C22" t="n">
         <v>7</v>
       </c>
       <c r="D22" t="n">
-        <v>37.62</v>
+        <v>39.62</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
         <v>2</v>
       </c>
       <c r="H22" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>High value</t>
+          <t>Middle</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B23" t="n">
-        <v>261</v>
+        <v>106</v>
       </c>
       <c r="C23" t="n">
         <v>7</v>
       </c>
       <c r="D23" t="n">
-        <v>47.62</v>
+        <v>38.62</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
         <v>2</v>
       </c>
-      <c r="G23" t="n">
-        <v>3</v>
-      </c>
       <c r="H23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -6155,28 +6155,28 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B24" t="n">
-        <v>186</v>
+        <v>79</v>
       </c>
       <c r="C24" t="n">
         <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>42.62</v>
+        <v>37.62</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6186,28 +6186,28 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B25" t="n">
+        <v>78</v>
+      </c>
+      <c r="C25" t="n">
+        <v>7</v>
+      </c>
+      <c r="D25" t="n">
+        <v>37.62</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="n">
         <v>5</v>
-      </c>
-      <c r="B25" t="n">
-        <v>230</v>
-      </c>
-      <c r="C25" t="n">
-        <v>7</v>
-      </c>
-      <c r="D25" t="n">
-        <v>40.62</v>
-      </c>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" t="n">
-        <v>6</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -6217,16 +6217,16 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B26" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C26" t="n">
         <v>7</v>
       </c>
       <c r="D26" t="n">
-        <v>39.62</v>
+        <v>37.62</v>
       </c>
       <c r="E26" t="n">
         <v>3</v>
@@ -6235,10 +6235,10 @@
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -6248,28 +6248,28 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="B27" t="n">
-        <v>447</v>
+        <v>18</v>
       </c>
       <c r="C27" t="n">
         <v>7</v>
       </c>
       <c r="D27" t="n">
-        <v>39.62</v>
+        <v>37.62</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -6279,28 +6279,28 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="B28" t="n">
-        <v>106</v>
+        <v>18</v>
       </c>
       <c r="C28" t="n">
         <v>7</v>
       </c>
       <c r="D28" t="n">
-        <v>38.62</v>
+        <v>37.62</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -6310,28 +6310,28 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>496</v>
+        <v>70</v>
       </c>
       <c r="C29" t="n">
         <v>7</v>
       </c>
       <c r="D29" t="n">
-        <v>38.62</v>
+        <v>37.62</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H29" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -6341,28 +6341,28 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>385</v>
+        <v>16</v>
       </c>
       <c r="C30" t="n">
         <v>7</v>
       </c>
       <c r="D30" t="n">
-        <v>38.62</v>
+        <v>37.62</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -6372,10 +6372,10 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B31" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C31" t="n">
         <v>7</v>
@@ -6387,13 +6387,13 @@
         <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
         <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -6403,10 +6403,10 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="B32" t="n">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="C32" t="n">
         <v>7</v>
@@ -6418,13 +6418,13 @@
         <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
         <v>1</v>
       </c>
       <c r="H32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -6434,10 +6434,10 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B33" t="n">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="C33" t="n">
         <v>7</v>
@@ -6449,13 +6449,13 @@
         <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -6465,10 +6465,10 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="B34" t="n">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="C34" t="n">
         <v>7</v>
@@ -6480,13 +6480,13 @@
         <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G34" t="n">
         <v>1</v>
       </c>
       <c r="H34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -6496,143 +6496,143 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="B35" t="n">
-        <v>13</v>
+        <v>509</v>
       </c>
       <c r="C35" t="n">
         <v>7</v>
       </c>
       <c r="D35" t="n">
-        <v>37.62</v>
+        <v>39.62</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
         <v>2</v>
       </c>
-      <c r="G35" t="n">
-        <v>1</v>
-      </c>
       <c r="H35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>292</v>
+        <v>447</v>
       </c>
       <c r="C36" t="n">
         <v>7</v>
       </c>
       <c r="D36" t="n">
-        <v>37.62</v>
+        <v>39.62</v>
       </c>
       <c r="E36" t="n">
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G36" t="n">
         <v>2</v>
       </c>
       <c r="H36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>53</v>
+        <v>15</v>
       </c>
       <c r="B37" t="n">
-        <v>341</v>
+        <v>372</v>
       </c>
       <c r="C37" t="n">
         <v>7</v>
       </c>
       <c r="D37" t="n">
-        <v>37.62</v>
+        <v>38.62</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
         <v>2</v>
       </c>
       <c r="H37" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="B38" t="n">
-        <v>478</v>
+        <v>465</v>
       </c>
       <c r="C38" t="n">
         <v>7</v>
       </c>
       <c r="D38" t="n">
-        <v>37.62</v>
+        <v>38.62</v>
       </c>
       <c r="E38" t="n">
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
       </c>
       <c r="H38" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="B39" t="n">
-        <v>137</v>
+        <v>496</v>
       </c>
       <c r="C39" t="n">
         <v>7</v>
       </c>
       <c r="D39" t="n">
-        <v>39.62</v>
+        <v>38.62</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
         <v>1</v>
@@ -6641,29 +6641,29 @@
         <v>2</v>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="B40" t="n">
-        <v>93</v>
+        <v>385</v>
       </c>
       <c r="C40" t="n">
         <v>7</v>
       </c>
       <c r="D40" t="n">
-        <v>39.62</v>
+        <v>38.62</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
         <v>1</v>
@@ -6672,51 +6672,51 @@
         <v>2</v>
       </c>
       <c r="H40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B41" t="n">
-        <v>509</v>
+        <v>132</v>
       </c>
       <c r="C41" t="n">
         <v>7</v>
       </c>
       <c r="D41" t="n">
-        <v>39.62</v>
+        <v>37.62</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B42" t="n">
-        <v>79</v>
+        <v>225</v>
       </c>
       <c r="C42" t="n">
         <v>7</v>
@@ -6725,7 +6725,7 @@
         <v>37.62</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>1</v>
@@ -6734,20 +6734,20 @@
         <v>1</v>
       </c>
       <c r="H42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B43" t="n">
-        <v>78</v>
+        <v>171</v>
       </c>
       <c r="C43" t="n">
         <v>7</v>
@@ -6756,7 +6756,7 @@
         <v>37.62</v>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
         <v>1</v>
@@ -6765,20 +6765,20 @@
         <v>1</v>
       </c>
       <c r="H43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="B44" t="n">
-        <v>75</v>
+        <v>163</v>
       </c>
       <c r="C44" t="n">
         <v>7</v>
@@ -6787,7 +6787,7 @@
         <v>37.62</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
         <v>1</v>
@@ -6796,20 +6796,20 @@
         <v>1</v>
       </c>
       <c r="H44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B45" t="n">
-        <v>163</v>
+        <v>109</v>
       </c>
       <c r="C45" t="n">
         <v>7</v>
@@ -6821,26 +6821,26 @@
         <v>2</v>
       </c>
       <c r="F45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G45" t="n">
         <v>1</v>
       </c>
       <c r="H45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="B46" t="n">
-        <v>109</v>
+        <v>248</v>
       </c>
       <c r="C46" t="n">
         <v>7</v>
@@ -6852,26 +6852,26 @@
         <v>2</v>
       </c>
       <c r="F46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46" t="n">
         <v>1</v>
       </c>
       <c r="H46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="B47" t="n">
-        <v>403</v>
+        <v>194</v>
       </c>
       <c r="C47" t="n">
         <v>7</v>
@@ -6880,29 +6880,29 @@
         <v>37.62</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="B48" t="n">
-        <v>540</v>
+        <v>140</v>
       </c>
       <c r="C48" t="n">
         <v>7</v>
@@ -6911,35 +6911,35 @@
         <v>37.62</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Middle</t>
+          <t>Low value</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B49" t="n">
-        <v>372</v>
+        <v>527</v>
       </c>
       <c r="C49" t="n">
         <v>7</v>
       </c>
       <c r="D49" t="n">
-        <v>38.62</v>
+        <v>37.62</v>
       </c>
       <c r="E49" t="n">
         <v>1</v>
@@ -6948,10 +6948,10 @@
         <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -6961,16 +6961,16 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B50" t="n">
-        <v>465</v>
+        <v>323</v>
       </c>
       <c r="C50" t="n">
         <v>7</v>
       </c>
       <c r="D50" t="n">
-        <v>38.62</v>
+        <v>37.62</v>
       </c>
       <c r="E50" t="n">
         <v>1</v>
@@ -6979,10 +6979,10 @@
         <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -6992,10 +6992,10 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B51" t="n">
-        <v>132</v>
+        <v>279</v>
       </c>
       <c r="C51" t="n">
         <v>7</v>
@@ -7004,7 +7004,7 @@
         <v>37.62</v>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
         <v>1</v>
@@ -7013,7 +7013,7 @@
         <v>1</v>
       </c>
       <c r="H51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -7023,10 +7023,10 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B52" t="n">
-        <v>225</v>
+        <v>416</v>
       </c>
       <c r="C52" t="n">
         <v>7</v>
@@ -7035,7 +7035,7 @@
         <v>37.62</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F52" t="n">
         <v>1</v>
@@ -7044,7 +7044,7 @@
         <v>1</v>
       </c>
       <c r="H52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -7054,10 +7054,10 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="B53" t="n">
-        <v>171</v>
+        <v>354</v>
       </c>
       <c r="C53" t="n">
         <v>7</v>
@@ -7066,7 +7066,7 @@
         <v>37.62</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
         <v>1</v>
@@ -7075,7 +7075,7 @@
         <v>1</v>
       </c>
       <c r="H53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -7085,10 +7085,10 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B54" t="n">
-        <v>354</v>
+        <v>310</v>
       </c>
       <c r="C54" t="n">
         <v>7</v>
@@ -7100,13 +7100,13 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G54" t="n">
         <v>1</v>
       </c>
       <c r="H54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -7116,10 +7116,10 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B55" t="n">
-        <v>310</v>
+        <v>403</v>
       </c>
       <c r="C55" t="n">
         <v>7</v>
@@ -7131,13 +7131,13 @@
         <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G55" t="n">
         <v>1</v>
       </c>
       <c r="H55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -7147,10 +7147,10 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="B56" t="n">
-        <v>527</v>
+        <v>540</v>
       </c>
       <c r="C56" t="n">
         <v>7</v>
@@ -7178,10 +7178,10 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="B57" t="n">
-        <v>323</v>
+        <v>292</v>
       </c>
       <c r="C57" t="n">
         <v>7</v>
@@ -7209,10 +7209,10 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="B58" t="n">
-        <v>279</v>
+        <v>341</v>
       </c>
       <c r="C58" t="n">
         <v>7</v>
@@ -7240,10 +7240,10 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="B59" t="n">
-        <v>416</v>
+        <v>478</v>
       </c>
       <c r="C59" t="n">
         <v>7</v>

</xml_diff>